<commit_message>
Push full codebase: exports, reports, dashboards, DBs, and docs
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/rlt_leave_report.xlsx
+++ b/rlt_leave_report.xlsx
@@ -7099,7 +7099,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Planned Leave</t>
+          <t>Resolved!</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -7124,13 +7124,13 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-03-07T13:23:13.421+0500</t>
+          <t>2026-03-09T13:34:46.951+0500</t>
         </is>
       </c>
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M86" t="n">
         <v>8</v>
@@ -28941,7 +28941,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Planned Leave</t>
+          <t>Resolved!</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -28966,13 +28966,13 @@
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>2026-03-07T13:23:13.421+0500</t>
+          <t>2026-03-09T13:34:46.951+0500</t>
         </is>
       </c>
       <c r="J204" t="inlineStr"/>
       <c r="K204" t="inlineStr"/>
       <c r="L204" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M204" t="n">
         <v>8</v>

</xml_diff>

<commit_message>
chore: push latest report snapshot before nested actual-hours fix
</commit_message>
<xml_diff>
--- a/rlt_leave_report.xlsx
+++ b/rlt_leave_report.xlsx
@@ -9402,7 +9402,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-03-16T10:29:39.119+0500</t>
+          <t>2026-03-24T14:47:00.468+0500</t>
         </is>
       </c>
       <c r="J108" t="inlineStr"/>
@@ -9411,7 +9411,7 @@
         <v>0</v>
       </c>
       <c r="M108" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="N108" t="inlineStr"/>
       <c r="O108" t="inlineStr">
@@ -9420,12 +9420,12 @@
         </is>
       </c>
       <c r="P108" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="Q108" t="inlineStr"/>
       <c r="R108" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="S108" t="inlineStr">
@@ -32210,7 +32210,7 @@
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>2026-03-16T10:29:39.119+0500</t>
+          <t>2026-03-24T14:47:00.468+0500</t>
         </is>
       </c>
       <c r="J226" t="inlineStr"/>
@@ -32219,7 +32219,7 @@
         <v>0</v>
       </c>
       <c r="M226" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="N226" t="inlineStr"/>
       <c r="O226" t="inlineStr">
@@ -32228,12 +32228,12 @@
         </is>
       </c>
       <c r="P226" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="Q226" t="inlineStr"/>
       <c r="R226" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="S226" t="inlineStr">
@@ -35771,7 +35771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E177"/>
+  <dimension ref="A1:E178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38804,37 +38804,37 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-215</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
+          <t>2026-03-03T09:00:00.000+0500</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Faiq Butt</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>RLT-202</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-03-04T04:41:00.000+0500</t>
+          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -38844,7 +38844,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Syed Yousaf Qadri</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -38854,12 +38854,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>RLT-208</t>
+          <t>RLT-202</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-03-04T14:27:00.000+0500</t>
+          <t>2026-03-04T04:41:00.000+0500</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -38869,7 +38869,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Ameer Hamza Khan</t>
+          <t>Syed Yousaf Qadri</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -38879,22 +38879,22 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-208</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
+          <t>2026-03-04T14:27:00.000+0500</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Ameer Hamza Khan</t>
         </is>
       </c>
       <c r="E125" t="n">
@@ -38904,12 +38904,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>RLT-209</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-03-05T14:27:00.000+0500</t>
+          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -38919,7 +38919,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Ameer Hamza Khan</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -38929,22 +38929,22 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-209</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
+          <t>2026-03-05T14:27:00.000+0500</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Ameer Hamza Khan</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -38954,12 +38954,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>RLT-203</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-03-06T09:00:00.000+0500</t>
+          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -38969,7 +38969,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Muhammad Abbas</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -38979,7 +38979,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>RLT-204</t>
+          <t>RLT-203</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -38994,22 +38994,22 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Zeeshan Sarwar</t>
+          <t>Muhammad Abbas</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>RLT-210</t>
+          <t>RLT-204</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-03-06T14:27:00.000+0500</t>
+          <t>2026-03-06T09:00:00.000+0500</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -39019,22 +39019,22 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Ameer Hamza Khan</t>
+          <t>Zeeshan Sarwar</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>RLT-213</t>
+          <t>RLT-210</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-03-06T09:00:00.000+0500</t>
+          <t>2026-03-06T14:27:00.000+0500</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -39044,7 +39044,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Faiq Butt</t>
+          <t>Ameer Hamza Khan</t>
         </is>
       </c>
       <c r="E131" t="n">
@@ -39054,22 +39054,22 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-213</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
+          <t>2026-03-06T09:00:00.000+0500</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Faiq Butt</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -39079,12 +39079,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>RLT-205</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-03-09T07:08:00.000+0500</t>
+          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -39094,22 +39094,22 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Sarmad Sabir</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="E133" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>RLT-214</t>
+          <t>RLT-205</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-03-09T09:00:00.000+0500</t>
+          <t>2026-03-09T07:08:00.000+0500</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -39119,47 +39119,47 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Faiq Butt</t>
+          <t>Sarmad Sabir</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>32</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-214</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
+          <t>2026-03-09T09:00:00.000+0500</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Faiq Butt</t>
         </is>
       </c>
       <c r="E135" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>RLT-211</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-03-10T14:28:00.000+0500</t>
+          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -39169,7 +39169,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Ameer Hamza Khan</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -39179,22 +39179,22 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-211</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
+          <t>2026-03-10T14:28:00.000+0500</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Ameer Hamza Khan</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -39214,7 +39214,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -39239,7 +39239,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -39254,12 +39254,12 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>RLT-212</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-03-13T09:00:00.000+0500</t>
+          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -39269,47 +39269,47 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Zeeshan Sarwar</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="E140" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-212</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
+          <t>2026-03-13T09:00:00.000+0500</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Zeeshan Sarwar</t>
         </is>
       </c>
       <c r="E141" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>RLT-216</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-03-16T09:00:00.000+0500</t>
+          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -39319,22 +39319,22 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Taimur Zahid</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="E142" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>RLT-218</t>
+          <t>RLT-216</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-03-16T15:30:00.000+0500</t>
+          <t>2026-03-16T09:00:00.000+0500</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -39344,7 +39344,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Arsalan Zafar Khan</t>
+          <t>Taimur Zahid</t>
         </is>
       </c>
       <c r="E143" t="n">
@@ -39354,37 +39354,37 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-218</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
+          <t>2026-03-16T15:30:00.000+0500</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Arsalan Zafar Khan</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>RLT-217</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-03-17T15:30:00.000+0500</t>
+          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -39394,36 +39394,36 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Muhammad Abdullah</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-217</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
+          <t>2026-03-17T15:30:00.000+0500</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Muhammad Abdullah</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="147">
@@ -39439,7 +39439,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -39464,7 +39464,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -39489,7 +39489,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -39514,7 +39514,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -39539,7 +39539,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -39564,7 +39564,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -39589,7 +39589,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -39614,7 +39614,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -39639,7 +39639,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -39654,17 +39654,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>RLT-173</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>redistributed:2026-04-01-&gt;2026-04-30</t>
+          <t>redistributed:2026-01-01-&gt;2026-03-31</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -39689,7 +39689,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -39714,7 +39714,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -39739,7 +39739,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -39764,7 +39764,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -39789,7 +39789,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -39814,7 +39814,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -39839,7 +39839,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -39864,7 +39864,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -39889,7 +39889,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -39914,7 +39914,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -39939,7 +39939,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -39964,7 +39964,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -39989,7 +39989,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -40014,7 +40014,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -40039,7 +40039,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -40064,7 +40064,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -40089,7 +40089,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -40114,7 +40114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -40139,7 +40139,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -40164,7 +40164,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -40189,15 +40189,40 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Maria Sharafat</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>RLT-173</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>redistributed:2026-04-01-&gt;2026-04-30</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="D177" t="inlineStr">
+      <c r="D178" t="inlineStr">
         <is>
           <t>Maria Sharafat</t>
         </is>
       </c>
-      <c r="E177" t="n">
+      <c r="E178" t="n">
         <v>8</v>
       </c>
     </row>
@@ -40424,7 +40449,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="C7" t="n">
         <v>30.5</v>
@@ -40439,7 +40464,7 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H7" t="n">
         <v>3.81</v>
@@ -40831,7 +40856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42273,7 +42298,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Hassan Malik</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -42282,7 +42307,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
@@ -42291,23 +42316,23 @@
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-215</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-215</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Muhammad Usman Javed</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -42316,10 +42341,10 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D44" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
@@ -42329,24 +42354,24 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>RLT-189</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-189</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ameer Hamza Khan</t>
+          <t>Muhammad Usman Javed</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -42363,19 +42388,19 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>RLT-208</t>
+          <t>RLT-189</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-208</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-189</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Hassan Malik</t>
+          <t>Ameer Hamza Khan</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -42397,19 +42422,19 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>RLT-202</t>
+          <t>RLT-208</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-202</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-208</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Hassan Malik</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -42418,10 +42443,10 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E47" t="n">
         <v>0</v>
@@ -42431,31 +42456,31 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-202</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-202</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ameer Hamza Khan</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D48" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E48" t="n">
         <v>0</v>
@@ -42465,19 +42490,19 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>RLT-209</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-209</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Ameer Hamza Khan</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -42486,10 +42511,10 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E49" t="n">
         <v>0</v>
@@ -42499,31 +42524,31 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-209</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-209</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ameer Hamza Khan</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D50" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
@@ -42533,19 +42558,19 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>RLT-210</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-210</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Hassan Malik</t>
+          <t>Ameer Hamza Khan</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -42557,29 +42582,29 @@
         <v>0</v>
       </c>
       <c r="D51" t="n">
-        <v>14.5</v>
+        <v>8</v>
       </c>
       <c r="E51" t="n">
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>14.5</v>
+        <v>8</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>RLT-204, RLT-213</t>
+          <t>RLT-210</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-204, https://octopusdtlsupport.atlassian.net/browse/RLT-213</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-210</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Hassan Malik</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -42588,32 +42613,32 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>14.5</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>8</v>
+        <v>14.5</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-204, RLT-213</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-204, https://octopusdtlsupport.atlassian.net/browse/RLT-213</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Muhammad Abbas</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -42622,10 +42647,10 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E53" t="n">
         <v>0</v>
@@ -42635,53 +42660,53 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>RLT-203</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-203</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Hassan Malik</t>
+          <t>Muhammad Abbas</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>RLT-214</t>
+          <t>RLT-203</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-214</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-203</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Hassan Malik</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -42690,7 +42715,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
@@ -42699,23 +42724,23 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-214</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-214</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Sarmad Sabir</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -42724,66 +42749,66 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D56" t="n">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="E56" t="n">
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>RLT-205</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-205</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ameer Hamza Khan</t>
+          <t>Sarmad Sabir</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="C57" t="n">
         <v>0</v>
       </c>
       <c r="D57" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="E57" t="n">
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>RLT-211</t>
+          <t>RLT-205</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-211</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-205</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Ameer Hamza Khan</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -42792,10 +42817,10 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E58" t="n">
         <v>0</v>
@@ -42805,12 +42830,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-211</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-211</t>
         </is>
       </c>
     </row>
@@ -42822,7 +42847,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -42856,7 +42881,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -42890,7 +42915,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -42919,41 +42944,41 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Arsalan Zafar Khan</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D62" t="n">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>RLT-218</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-218</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Arsalan Zafar Khan</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -42962,32 +42987,32 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="E63" t="n">
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-218</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-218</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Taimur Zahid</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -42996,66 +43021,66 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D64" t="n">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="E64" t="n">
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>RLT-216</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-216</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Taimur Zahid</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="E65" t="n">
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-216</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-216</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Muhammad Abdullah</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -43064,59 +43089,59 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D66" t="n">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="E66" t="n">
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>RLT-217</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-217</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Muhammad Abdullah</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="E67" t="n">
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-217</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-217</t>
         </is>
       </c>
     </row>
@@ -43128,7 +43153,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -43162,7 +43187,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -43196,7 +43221,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -43230,7 +43255,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -43264,7 +43289,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -43298,7 +43323,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -43332,7 +43357,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -43366,7 +43391,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -43400,7 +43425,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -43434,7 +43459,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -43451,19 +43476,19 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>RLT-173</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-173</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-172</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Muhammad Imran Aslam</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -43472,59 +43497,59 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D78" t="n">
         <v>0</v>
       </c>
       <c r="E78" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F78" t="n">
         <v>8</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>RLT-176</t>
+          <t>RLT-173</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-176</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-173</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Muhammad Imran Aslam</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D79" t="n">
         <v>0</v>
       </c>
       <c r="E79" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F79" t="n">
         <v>8</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>RLT-173</t>
+          <t>RLT-176</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-173</t>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-176</t>
         </is>
       </c>
     </row>
@@ -43536,7 +43561,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -43570,7 +43595,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -43604,7 +43629,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -43638,7 +43663,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -43672,7 +43697,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -43706,7 +43731,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -43740,7 +43765,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -43774,7 +43799,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -43808,7 +43833,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -43842,7 +43867,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -43876,7 +43901,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -43910,7 +43935,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -43944,7 +43969,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -43978,7 +44003,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -44012,7 +44037,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -44046,7 +44071,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -44080,7 +44105,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -44114,7 +44139,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -44148,7 +44173,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -44182,27 +44207,61 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>8</v>
+      </c>
+      <c r="D99" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" t="n">
+        <v>8</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>RLT-173</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://octopusdtlsupport.atlassian.net/browse/RLT-173</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Maria Sharafat</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="C99" t="n">
-        <v>8</v>
-      </c>
-      <c r="D99" t="n">
-        <v>0</v>
-      </c>
-      <c r="E99" t="n">
-        <v>0</v>
-      </c>
-      <c r="F99" t="n">
-        <v>8</v>
-      </c>
-      <c r="G99" t="inlineStr">
+      <c r="C100" t="n">
+        <v>8</v>
+      </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" t="n">
+        <v>8</v>
+      </c>
+      <c r="G100" t="inlineStr">
         <is>
           <t>RLT-173</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr">
+      <c r="H100" t="inlineStr">
         <is>
           <t>https://octopusdtlsupport.atlassian.net/browse/RLT-173</t>
         </is>
@@ -44674,7 +44733,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="D19" t="n">
         <v>22.5</v>
@@ -44683,7 +44742,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>22.5</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="20">
@@ -45536,7 +45595,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="D15" t="n">
         <v>22.5</v>
@@ -45545,7 +45604,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>54.5</v>
+        <v>78.5</v>
       </c>
     </row>
     <row r="16">
@@ -46877,7 +46936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47102,17 +47161,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RLT-116</t>
+          <t>RLT-215</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hassan Saeed Wattoo</t>
+          <t>Hassan Malik</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Annual Leaves</t>
+          <t>Compassionate Leaves</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -47122,11 +47181,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Planned Leave</t>
+          <t>Considered in Roadmap &amp; Queued</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -47145,7 +47204,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RLT-65</t>
+          <t>RLT-116</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -47155,7 +47214,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Annual Leave 23rd Dec, 24th Dec, 26th Dec, 27th Dec</t>
+          <t>Annual Leaves</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -47169,7 +47228,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -47188,7 +47247,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RLT-89</t>
+          <t>RLT-65</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -47198,21 +47257,21 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Compassionate Leave 29th Sept, 30th Sept, 1st Oct</t>
+          <t>Annual Leave 23rd Dec, 24th Dec, 26th Dec, 27th Dec</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Unplanned</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Emergency Leave</t>
+          <t>Planned Leave</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -47231,7 +47290,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RLT-96</t>
+          <t>RLT-89</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -47241,7 +47300,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Compassionate Leaves 24th Nov, 25th Nov 2025</t>
+          <t>Compassionate Leave 29th Sept, 30th Sept, 1st Oct</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -47255,7 +47314,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -47274,50 +47333,50 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RLT-172</t>
+          <t>RLT-96</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Maria Sharafat</t>
+          <t>Hassan Saeed Wattoo</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Maternity Leaves 1 Jan - 31 March 2026</t>
+          <t>Compassionate Leaves 24th Nov, 25th Nov 2025</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Unplanned</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Considered in Roadmap &amp; Queued</t>
+          <t>Emergency Leave</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>528</v>
+        <v>16</v>
       </c>
       <c r="G10" t="n">
-        <v>528</v>
+        <v>0</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>No Entry</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>No Entry</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RLT-173</t>
+          <t>RLT-172</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -47327,7 +47386,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Annual Leaves 1 April - 30 April 2026</t>
+          <t>Maternity Leaves 1 Jan - 31 March 2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -47341,36 +47400,36 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>176</v>
+        <v>528</v>
       </c>
       <c r="G11" t="n">
-        <v>176</v>
+        <v>528</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RLT-188</t>
+          <t>RLT-173</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Muhammad Usman Javed</t>
+          <t>Maria Sharafat</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Annual Leaves</t>
+          <t>Annual Leaves 1 April - 30 April 2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -47384,60 +47443,103 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>56</v>
+        <v>176</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>176</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>No Entry</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>No Entry</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>RLT-188</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Muhammad Usman Javed</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Annual Leaves</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Considered in Roadmap &amp; Queued</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>56</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>No Entry</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>No Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>RLT-47</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Zeeshan Sarwar</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Leave for two days 20 and 21-06-24</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Resolved!</t>
         </is>
       </c>
-      <c r="F13" t="n">
+      <c r="F14" t="n">
         <v>16</v>
       </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="inlineStr">
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>No Entry</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>No Entry</t>
         </is>

</xml_diff>